<commit_message>
statistical study updated to check the normality of the data
</commit_message>
<xml_diff>
--- a/logs/final_winner_optimization/experiments_summary.xlsx
+++ b/logs/final_winner_optimization/experiments_summary.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BW47"/>
+  <dimension ref="A1:BW50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12997,6 +12997,801 @@
       </c>
       <c r="BW47" t="n">
         <v>-0.1203773281354161</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>46085.59322916667</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>03-04_14-14-15_multihead_spsa_compact_f5_w5_h5_effsu2_effsu2_realamplitudes_full_r2_3_2.pkl</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Final (Last Iteration)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>data/reduce_row_number_absolutes</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>16590</v>
+      </c>
+      <c r="G48" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>[['wv', 'sv', 'rarad'], ['sv', 'yr', 'rarad'], ['ya', 'yr']]</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>['Surge Velocity', 'Sway Velocity', 'Yaw Rate', 'Yaw Angle']</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>5</v>
+      </c>
+      <c r="K48" t="n">
+        <v>5</v>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>motion</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>multihead</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]</t>
+        </is>
+      </c>
+      <c r="R48" t="n">
+        <v>3</v>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>compact</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>['effsu2', 'effsu2', 'realamplitudes']</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>[2, 3, 2]</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>[[0, 1, 2], [0, 1, 2], [0, 1, -1]]</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>spsa</t>
+        </is>
+      </c>
+      <c r="Z48" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AA48" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AB48" t="inlineStr"/>
+      <c r="AC48" t="n">
+        <v>512</v>
+      </c>
+      <c r="AD48" t="inlineStr">
+        <is>
+          <t>[0.05, 0.0001]</t>
+        </is>
+      </c>
+      <c r="AE48" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AF48" t="n">
+        <v>180</v>
+      </c>
+      <c r="AG48" t="n">
+        <v>60</v>
+      </c>
+      <c r="AH48" t="n">
+        <v>120</v>
+      </c>
+      <c r="AI48" t="n">
+        <v>0.0688618667531352</v>
+      </c>
+      <c r="AJ48" t="n">
+        <v>9.583562204354951</v>
+      </c>
+      <c r="AK48" t="n">
+        <v>0.7895707621960872</v>
+      </c>
+      <c r="AL48" t="n">
+        <v>0.1867260167949384</v>
+      </c>
+      <c r="AM48" t="n">
+        <v>11.95718005622282</v>
+      </c>
+      <c r="AN48" t="n">
+        <v>0.7981323573928729</v>
+      </c>
+      <c r="AO48" t="n">
+        <v>11.95718005622282</v>
+      </c>
+      <c r="AP48" t="n">
+        <v>11.95718005622282</v>
+      </c>
+      <c r="AQ48" t="n">
+        <v>0.7981323573928729</v>
+      </c>
+      <c r="AR48" t="n">
+        <v>71.91863557898208</v>
+      </c>
+      <c r="AS48" t="n">
+        <v>0.2530134619383231</v>
+      </c>
+      <c r="AT48" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AU48" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
+      <c r="AV48" t="n">
+        <v>0.04296638765079115</v>
+      </c>
+      <c r="AW48" t="n">
+        <v>0.6880084718975934</v>
+      </c>
+      <c r="AX48" t="n">
+        <v>0.04296638765079115</v>
+      </c>
+      <c r="AY48" t="n">
+        <v>0.04296638765079115</v>
+      </c>
+      <c r="AZ48" t="n">
+        <v>0.6880084718975934</v>
+      </c>
+      <c r="BA48" t="n">
+        <v>0.1035975684120596</v>
+      </c>
+      <c r="BB48" t="n">
+        <v>0.2477477059680875</v>
+      </c>
+      <c r="BC48" t="n">
+        <v>0.03498156467388404</v>
+      </c>
+      <c r="BD48" t="n">
+        <v>0.8787963498379168</v>
+      </c>
+      <c r="BE48" t="n">
+        <v>0.03498156467388404</v>
+      </c>
+      <c r="BF48" t="n">
+        <v>0.03498156467388404</v>
+      </c>
+      <c r="BG48" t="n">
+        <v>0.8787963498379168</v>
+      </c>
+      <c r="BH48" t="n">
+        <v>0.2109588777335622</v>
+      </c>
+      <c r="BI48" t="n">
+        <v>0.2690725456745151</v>
+      </c>
+      <c r="BJ48" t="n">
+        <v>0.05941623395545763</v>
+      </c>
+      <c r="BK48" t="n">
+        <v>0.7614626141368163</v>
+      </c>
+      <c r="BL48" t="n">
+        <v>0.05941623395545763</v>
+      </c>
+      <c r="BM48" t="n">
+        <v>0.05941623395545763</v>
+      </c>
+      <c r="BN48" t="n">
+        <v>0.7614626141368163</v>
+      </c>
+      <c r="BO48" t="n">
+        <v>0.1712156149531613</v>
+      </c>
+      <c r="BP48" t="n">
+        <v>0.3126234617882054</v>
+      </c>
+      <c r="BQ48" t="n">
+        <v>47.69135603861108</v>
+      </c>
+      <c r="BR48" t="n">
+        <v>0.8642619936991655</v>
+      </c>
+      <c r="BS48" t="n">
+        <v>47.69135603861108</v>
+      </c>
+      <c r="BT48" t="n">
+        <v>47.69135603861108</v>
+      </c>
+      <c r="BU48" t="n">
+        <v>0.8642619936991655</v>
+      </c>
+      <c r="BV48" t="n">
+        <v>287.18877025483</v>
+      </c>
+      <c r="BW48" t="n">
+        <v>0.182610134322481</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>46085.88435185186</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>03-04_21-13-28_multihead_spsa_compact_f5_w5_h5_effsu2_effsu2_realamplitudes_full_r2_3_2.pkl</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>3</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Best (Lowest Val Loss)</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>data/reduce_row_number_absolutes</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>16590</v>
+      </c>
+      <c r="G49" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>[['wv', 'sv', 'rarad'], ['sv', 'yr', 'rarad'], ['ya', 'yr']]</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>['Surge Velocity', 'Sway Velocity', 'Yaw Rate', 'Yaw Angle']</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>5</v>
+      </c>
+      <c r="K49" t="n">
+        <v>5</v>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>motion</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>multihead</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]</t>
+        </is>
+      </c>
+      <c r="R49" t="n">
+        <v>3</v>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>compact</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>['effsu2', 'effsu2', 'realamplitudes']</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>[2, 3, 2]</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>[[0, 1, 2], [0, 1, 2], [0, 1, -1]]</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>spsa</t>
+        </is>
+      </c>
+      <c r="Z49" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AA49" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AB49" t="inlineStr"/>
+      <c r="AC49" t="n">
+        <v>512</v>
+      </c>
+      <c r="AD49" t="inlineStr">
+        <is>
+          <t>[0.05, 0.0001]</t>
+        </is>
+      </c>
+      <c r="AE49" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AF49" t="n">
+        <v>180</v>
+      </c>
+      <c r="AG49" t="n">
+        <v>60</v>
+      </c>
+      <c r="AH49" t="n">
+        <v>120</v>
+      </c>
+      <c r="AI49" t="n">
+        <v>0.07419820570411019</v>
+      </c>
+      <c r="AJ49" t="n">
+        <v>12.96923574920233</v>
+      </c>
+      <c r="AK49" t="n">
+        <v>0.7578659912293069</v>
+      </c>
+      <c r="AL49" t="n">
+        <v>-0.2555740921623109</v>
+      </c>
+      <c r="AM49" t="n">
+        <v>15.77922734055479</v>
+      </c>
+      <c r="AN49" t="n">
+        <v>0.7697312645606686</v>
+      </c>
+      <c r="AO49" t="n">
+        <v>15.77922734055479</v>
+      </c>
+      <c r="AP49" t="n">
+        <v>15.77922734055479</v>
+      </c>
+      <c r="AQ49" t="n">
+        <v>0.7697312645606686</v>
+      </c>
+      <c r="AR49" t="n">
+        <v>118.4743665401534</v>
+      </c>
+      <c r="AS49" t="n">
+        <v>-0.1491931009169778</v>
+      </c>
+      <c r="AT49" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AU49" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
+      <c r="AV49" t="n">
+        <v>0.06134868607458734</v>
+      </c>
+      <c r="AW49" t="n">
+        <v>0.5545292177911795</v>
+      </c>
+      <c r="AX49" t="n">
+        <v>0.06134868607458734</v>
+      </c>
+      <c r="AY49" t="n">
+        <v>0.06134868607458734</v>
+      </c>
+      <c r="AZ49" t="n">
+        <v>0.5545292177911795</v>
+      </c>
+      <c r="BA49" t="n">
+        <v>0.2309898427035444</v>
+      </c>
+      <c r="BB49" t="n">
+        <v>-0.6772849183165248</v>
+      </c>
+      <c r="BC49" t="n">
+        <v>0.03319135360437299</v>
+      </c>
+      <c r="BD49" t="n">
+        <v>0.8849990488368925</v>
+      </c>
+      <c r="BE49" t="n">
+        <v>0.03319135360437299</v>
+      </c>
+      <c r="BF49" t="n">
+        <v>0.03319135360437299</v>
+      </c>
+      <c r="BG49" t="n">
+        <v>0.8849990488368925</v>
+      </c>
+      <c r="BH49" t="n">
+        <v>0.2188420949913155</v>
+      </c>
+      <c r="BI49" t="n">
+        <v>0.2417588815897939</v>
+      </c>
+      <c r="BJ49" t="n">
+        <v>0.04517392211113919</v>
+      </c>
+      <c r="BK49" t="n">
+        <v>0.818640991321389</v>
+      </c>
+      <c r="BL49" t="n">
+        <v>0.04517392211113919</v>
+      </c>
+      <c r="BM49" t="n">
+        <v>0.04517392211113919</v>
+      </c>
+      <c r="BN49" t="n">
+        <v>0.818640991321389</v>
+      </c>
+      <c r="BO49" t="n">
+        <v>0.2028324767243428</v>
+      </c>
+      <c r="BP49" t="n">
+        <v>0.1856917622505154</v>
+      </c>
+      <c r="BQ49" t="n">
+        <v>62.977195400429</v>
+      </c>
+      <c r="BR49" t="n">
+        <v>0.8207558002932123</v>
+      </c>
+      <c r="BS49" t="n">
+        <v>62.977195400429</v>
+      </c>
+      <c r="BT49" t="n">
+        <v>62.977195400429</v>
+      </c>
+      <c r="BU49" t="n">
+        <v>0.8207558002932123</v>
+      </c>
+      <c r="BV49" t="n">
+        <v>473.2448017461955</v>
+      </c>
+      <c r="BW49" t="n">
+        <v>-0.3469381291917044</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46086.14479166667</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>03-05_03-28-30_multihead_spsa_compact_f5_w5_h5_effsu2_effsu2_realamplitudes_full_r2_3_2.pkl</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Best (Lowest Val Loss)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>data/reduce_row_number_absolutes</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>16590</v>
+      </c>
+      <c r="G50" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>[['wv', 'sv', 'rarad'], ['sv', 'yr', 'rarad'], ['ya', 'yr']]</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>['Surge Velocity', 'Sway Velocity', 'Yaw Rate', 'Yaw Angle']</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>5</v>
+      </c>
+      <c r="K50" t="n">
+        <v>5</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>motion</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>multihead</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>[{'features': ['wv', 'sv', 'rarad'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['sv', 'yr', 'rarad'], 'output_dim': 2, 'reps': 3, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'full', 'map': [0, 1, 2]}, {'features': ['ya', 'yr'], 'output_dim': 1, 'reps': 2, 'encoding': 'compact', 'ansatz': 'realamplitudes', 'entangle': 'full', 'map': [0, 1, -1]}]</t>
+        </is>
+      </c>
+      <c r="R50" t="n">
+        <v>3</v>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>compact</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>['effsu2', 'effsu2', 'realamplitudes']</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>[2, 3, 2]</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>[[0, 1, 2], [0, 1, 2], [0, 1, -1]]</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>spsa</t>
+        </is>
+      </c>
+      <c r="Z50" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AA50" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AB50" t="inlineStr"/>
+      <c r="AC50" t="n">
+        <v>512</v>
+      </c>
+      <c r="AD50" t="inlineStr">
+        <is>
+          <t>[0.05, 0.0001]</t>
+        </is>
+      </c>
+      <c r="AE50" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AF50" t="n">
+        <v>180</v>
+      </c>
+      <c r="AG50" t="n">
+        <v>60</v>
+      </c>
+      <c r="AH50" t="n">
+        <v>120</v>
+      </c>
+      <c r="AI50" t="n">
+        <v>0.07900416701343374</v>
+      </c>
+      <c r="AJ50" t="n">
+        <v>11.40153630673874</v>
+      </c>
+      <c r="AK50" t="n">
+        <v>0.7555643148997051</v>
+      </c>
+      <c r="AL50" t="n">
+        <v>-0.147127665579905</v>
+      </c>
+      <c r="AM50" t="n">
+        <v>19.9078231520243</v>
+      </c>
+      <c r="AN50" t="n">
+        <v>0.7283214983078622</v>
+      </c>
+      <c r="AO50" t="n">
+        <v>19.9078231520243</v>
+      </c>
+      <c r="AP50" t="n">
+        <v>19.9078231520243</v>
+      </c>
+      <c r="AQ50" t="n">
+        <v>0.7283214983078622</v>
+      </c>
+      <c r="AR50" t="n">
+        <v>98.11610278894445</v>
+      </c>
+      <c r="AS50" t="n">
+        <v>-0.02310761739814438</v>
+      </c>
+      <c r="AT50" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AU50" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
+      <c r="AV50" t="n">
+        <v>0.05284324896903466</v>
+      </c>
+      <c r="AW50" t="n">
+        <v>0.6162896883549978</v>
+      </c>
+      <c r="AX50" t="n">
+        <v>0.05284324896903466</v>
+      </c>
+      <c r="AY50" t="n">
+        <v>0.05284324896903466</v>
+      </c>
+      <c r="AZ50" t="n">
+        <v>0.6162896883549978</v>
+      </c>
+      <c r="BA50" t="n">
+        <v>0.2841851157132149</v>
+      </c>
+      <c r="BB50" t="n">
+        <v>-1.063551379649031</v>
+      </c>
+      <c r="BC50" t="n">
+        <v>0.04933045706436691</v>
+      </c>
+      <c r="BD50" t="n">
+        <v>0.8290805023701835</v>
+      </c>
+      <c r="BE50" t="n">
+        <v>0.04933045706436691</v>
+      </c>
+      <c r="BF50" t="n">
+        <v>0.04933045706436691</v>
+      </c>
+      <c r="BG50" t="n">
+        <v>0.8290805023701835</v>
+      </c>
+      <c r="BH50" t="n">
+        <v>0.1303605701015614</v>
+      </c>
+      <c r="BI50" t="n">
+        <v>0.5483284672707845</v>
+      </c>
+      <c r="BJ50" t="n">
+        <v>0.07620705077703777</v>
+      </c>
+      <c r="BK50" t="n">
+        <v>0.6940527955655165</v>
+      </c>
+      <c r="BL50" t="n">
+        <v>0.07620705077703777</v>
+      </c>
+      <c r="BM50" t="n">
+        <v>0.07620705077703777</v>
+      </c>
+      <c r="BN50" t="n">
+        <v>0.6940527955655165</v>
+      </c>
+      <c r="BO50" t="n">
+        <v>0.1150008012961386</v>
+      </c>
+      <c r="BP50" t="n">
+        <v>0.5383081577685118</v>
+      </c>
+      <c r="BQ50" t="n">
+        <v>79.4529118512866</v>
+      </c>
+      <c r="BR50" t="n">
+        <v>0.7738630069407504</v>
+      </c>
+      <c r="BS50" t="n">
+        <v>79.4529118512866</v>
+      </c>
+      <c r="BT50" t="n">
+        <v>79.4529118512866</v>
+      </c>
+      <c r="BU50" t="n">
+        <v>0.7738630069407504</v>
+      </c>
+      <c r="BV50" t="n">
+        <v>391.9348646686658</v>
+      </c>
+      <c r="BW50" t="n">
+        <v>-0.1155157149828334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>